<commit_message>
Fix stale binyan-1 hardcoded forms in xlsx practice sheets
Sheets "תרגול פעלים" and "פתרונות" (rows 502-551) still had the 50
binyan-1 practice forms as hardcoded text generated by the old buggy
engine. Regenerated all 50 via the now-fixed VerbEngine and overwrote
only the "הפועל" column, matched by (root, tense, person) - 19 of 50
actually changed value; the other 31 already happened to match since
that root's relevant vowel was "a". No other column, row, or sheet
touched.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/אוצר_מילים_ערבית.xlsx
+++ b/אוצר_מילים_ערבית.xlsx
@@ -20770,7 +20770,7 @@
     <row r="505">
       <c r="A505" s="10" t="inlineStr">
         <is>
-          <t>شَرَبَ</t>
+          <t>شَرِبَ</t>
         </is>
       </c>
       <c r="B505" s="11" t="n"/>
@@ -20794,7 +20794,7 @@
     <row r="507">
       <c r="A507" s="10" t="inlineStr">
         <is>
-          <t>اِرْجَعْ</t>
+          <t>اِرْجِعْ</t>
         </is>
       </c>
       <c r="B507" s="11" t="n"/>
@@ -20818,7 +20818,7 @@
     <row r="509">
       <c r="A509" s="10" t="inlineStr">
         <is>
-          <t>تَدْخَلُونَ</t>
+          <t>تَدْخُلُونَ</t>
         </is>
       </c>
       <c r="B509" s="11" t="n"/>
@@ -20830,7 +20830,7 @@
     <row r="510">
       <c r="A510" s="10" t="inlineStr">
         <is>
-          <t>اِجْلَسُوا</t>
+          <t>اِجْلِسُوا</t>
         </is>
       </c>
       <c r="B510" s="11" t="n"/>
@@ -20902,7 +20902,7 @@
     <row r="516">
       <c r="A516" s="10" t="inlineStr">
         <is>
-          <t>اِغْلَقْنَ</t>
+          <t>اِغْلِقْنَ</t>
         </is>
       </c>
       <c r="B516" s="11" t="n"/>
@@ -20926,7 +20926,7 @@
     <row r="518">
       <c r="A518" s="10" t="inlineStr">
         <is>
-          <t>يَعْرَفُ</t>
+          <t>يَعْرِفُ</t>
         </is>
       </c>
       <c r="B518" s="11" t="n"/>
@@ -20962,7 +20962,7 @@
     <row r="521">
       <c r="A521" s="10" t="inlineStr">
         <is>
-          <t>تَغْسَلَانِ</t>
+          <t>تَغْسِلَانِ</t>
         </is>
       </c>
       <c r="B521" s="11" t="n"/>
@@ -20986,7 +20986,7 @@
     <row r="523">
       <c r="A523" s="10" t="inlineStr">
         <is>
-          <t>رَكَبْتُنَّ</t>
+          <t>رَكِبْتُنَّ</t>
         </is>
       </c>
       <c r="B523" s="11" t="n"/>
@@ -20998,7 +20998,7 @@
     <row r="524">
       <c r="A524" s="10" t="inlineStr">
         <is>
-          <t>يَنْزَلَانِ</t>
+          <t>يَنْزِلَانِ</t>
         </is>
       </c>
       <c r="B524" s="11" t="n"/>
@@ -21034,7 +21034,7 @@
     <row r="527">
       <c r="A527" s="10" t="inlineStr">
         <is>
-          <t>يَرْسَمْنَ</t>
+          <t>يَرْسُمْنَ</t>
         </is>
       </c>
       <c r="B527" s="11" t="n"/>
@@ -21046,7 +21046,7 @@
     <row r="528">
       <c r="A528" s="10" t="inlineStr">
         <is>
-          <t>اِطْبَخِي</t>
+          <t>اُطْبُخِي</t>
         </is>
       </c>
       <c r="B528" s="11" t="n"/>
@@ -21070,7 +21070,7 @@
     <row r="530">
       <c r="A530" s="10" t="inlineStr">
         <is>
-          <t>تَحْمَلِينَ</t>
+          <t>تَحْمِلِينَ</t>
         </is>
       </c>
       <c r="B530" s="11" t="n"/>
@@ -21118,7 +21118,7 @@
     <row r="534">
       <c r="A534" s="10" t="inlineStr">
         <is>
-          <t>اِضْرَبَا</t>
+          <t>اِضْرِبَا</t>
         </is>
       </c>
       <c r="B534" s="11" t="n"/>
@@ -21190,7 +21190,7 @@
     <row r="540">
       <c r="A540" s="10" t="inlineStr">
         <is>
-          <t>اِقْفَزُوا</t>
+          <t>اِقْفِزُوا</t>
         </is>
       </c>
       <c r="B540" s="11" t="n"/>
@@ -21214,7 +21214,7 @@
     <row r="542">
       <c r="A542" s="10" t="inlineStr">
         <is>
-          <t>تَكْتَبُ</t>
+          <t>تَكْتُبُ</t>
         </is>
       </c>
       <c r="B542" s="11" t="n"/>
@@ -21238,7 +21238,7 @@
     <row r="544">
       <c r="A544" s="10" t="inlineStr">
         <is>
-          <t>سَمَعَ</t>
+          <t>سَمِعَ</t>
         </is>
       </c>
       <c r="B544" s="11" t="n"/>
@@ -21286,7 +21286,7 @@
     <row r="548">
       <c r="A548" s="10" t="inlineStr">
         <is>
-          <t>تَخْرَجُونَ</t>
+          <t>تَخْرُجُونَ</t>
         </is>
       </c>
       <c r="B548" s="11" t="n"/>
@@ -21298,7 +21298,7 @@
     <row r="549">
       <c r="A549" s="10" t="inlineStr">
         <is>
-          <t>اِدْخَلَا</t>
+          <t>اُدْخُلَا</t>
         </is>
       </c>
       <c r="B549" s="11" t="n"/>
@@ -21322,7 +21322,7 @@
     <row r="551">
       <c r="A551" s="10" t="inlineStr">
         <is>
-          <t>تَنْظَرَانِ</t>
+          <t>تَنْظُرَانِ</t>
         </is>
       </c>
       <c r="B551" s="11" t="n"/>
@@ -37484,7 +37484,7 @@
     <row r="505">
       <c r="A505" s="10" t="inlineStr">
         <is>
-          <t>شَرَبَ</t>
+          <t>شَرِبَ</t>
         </is>
       </c>
       <c r="B505" s="10" t="inlineStr">
@@ -37548,7 +37548,7 @@
     <row r="507">
       <c r="A507" s="10" t="inlineStr">
         <is>
-          <t>اِرْجَعْ</t>
+          <t>اِرْجِعْ</t>
         </is>
       </c>
       <c r="B507" s="10" t="inlineStr">
@@ -37612,7 +37612,7 @@
     <row r="509">
       <c r="A509" s="10" t="inlineStr">
         <is>
-          <t>تَدْخَلُونَ</t>
+          <t>تَدْخُلُونَ</t>
         </is>
       </c>
       <c r="B509" s="10" t="inlineStr">
@@ -37644,7 +37644,7 @@
     <row r="510">
       <c r="A510" s="10" t="inlineStr">
         <is>
-          <t>اِجْلَسُوا</t>
+          <t>اِجْلِسُوا</t>
         </is>
       </c>
       <c r="B510" s="10" t="inlineStr">
@@ -37836,7 +37836,7 @@
     <row r="516">
       <c r="A516" s="10" t="inlineStr">
         <is>
-          <t>اِغْلَقْنَ</t>
+          <t>اِغْلِقْنَ</t>
         </is>
       </c>
       <c r="B516" s="10" t="inlineStr">
@@ -37900,7 +37900,7 @@
     <row r="518">
       <c r="A518" s="10" t="inlineStr">
         <is>
-          <t>يَعْرَفُ</t>
+          <t>يَعْرِفُ</t>
         </is>
       </c>
       <c r="B518" s="10" t="inlineStr">
@@ -37996,7 +37996,7 @@
     <row r="521">
       <c r="A521" s="10" t="inlineStr">
         <is>
-          <t>تَغْسَلَانِ</t>
+          <t>تَغْسِلَانِ</t>
         </is>
       </c>
       <c r="B521" s="10" t="inlineStr">
@@ -38060,7 +38060,7 @@
     <row r="523">
       <c r="A523" s="10" t="inlineStr">
         <is>
-          <t>رَكَبْتُنَّ</t>
+          <t>رَكِبْتُنَّ</t>
         </is>
       </c>
       <c r="B523" s="10" t="inlineStr">
@@ -38092,7 +38092,7 @@
     <row r="524">
       <c r="A524" s="10" t="inlineStr">
         <is>
-          <t>يَنْزَلَانِ</t>
+          <t>يَنْزِلَانِ</t>
         </is>
       </c>
       <c r="B524" s="10" t="inlineStr">
@@ -38188,7 +38188,7 @@
     <row r="527">
       <c r="A527" s="10" t="inlineStr">
         <is>
-          <t>يَرْسَمْنَ</t>
+          <t>يَرْسُمْنَ</t>
         </is>
       </c>
       <c r="B527" s="10" t="inlineStr">
@@ -38220,7 +38220,7 @@
     <row r="528">
       <c r="A528" s="10" t="inlineStr">
         <is>
-          <t>اِطْبَخِي</t>
+          <t>اُطْبُخِي</t>
         </is>
       </c>
       <c r="B528" s="10" t="inlineStr">
@@ -38284,7 +38284,7 @@
     <row r="530">
       <c r="A530" s="10" t="inlineStr">
         <is>
-          <t>تَحْمَلِينَ</t>
+          <t>تَحْمِلِينَ</t>
         </is>
       </c>
       <c r="B530" s="10" t="inlineStr">
@@ -38412,7 +38412,7 @@
     <row r="534">
       <c r="A534" s="10" t="inlineStr">
         <is>
-          <t>اِضْرَبَا</t>
+          <t>اِضْرِبَا</t>
         </is>
       </c>
       <c r="B534" s="10" t="inlineStr">
@@ -38604,7 +38604,7 @@
     <row r="540">
       <c r="A540" s="10" t="inlineStr">
         <is>
-          <t>اِقْفَزُوا</t>
+          <t>اِقْفِزُوا</t>
         </is>
       </c>
       <c r="B540" s="10" t="inlineStr">
@@ -38668,7 +38668,7 @@
     <row r="542">
       <c r="A542" s="10" t="inlineStr">
         <is>
-          <t>تَكْتَبُ</t>
+          <t>تَكْتُبُ</t>
         </is>
       </c>
       <c r="B542" s="10" t="inlineStr">
@@ -38732,7 +38732,7 @@
     <row r="544">
       <c r="A544" s="10" t="inlineStr">
         <is>
-          <t>سَمَعَ</t>
+          <t>سَمِعَ</t>
         </is>
       </c>
       <c r="B544" s="10" t="inlineStr">
@@ -38860,7 +38860,7 @@
     <row r="548">
       <c r="A548" s="10" t="inlineStr">
         <is>
-          <t>تَخْرَجُونَ</t>
+          <t>تَخْرُجُونَ</t>
         </is>
       </c>
       <c r="B548" s="10" t="inlineStr">
@@ -38892,7 +38892,7 @@
     <row r="549">
       <c r="A549" s="10" t="inlineStr">
         <is>
-          <t>اِدْخَلَا</t>
+          <t>اُدْخُلَا</t>
         </is>
       </c>
       <c r="B549" s="10" t="inlineStr">
@@ -38956,7 +38956,7 @@
     <row r="551">
       <c r="A551" s="10" t="inlineStr">
         <is>
-          <t>تَنْظَرَانِ</t>
+          <t>تَنْظُرَانِ</t>
         </is>
       </c>
       <c r="B551" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Revert "Add vocalized Arabic (arabicVoc) for chapter 1, infrastructure for the rest"
This reverts commit 2786cdf8bec18d5dcd2c9a4af13b79303a13b009.
</commit_message>
<xml_diff>
--- a/אוצר_מילים_ערבית.xlsx
+++ b/אוצר_מילים_ערבית.xlsx
@@ -506,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F403"/>
+  <dimension ref="A1:E403"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="9" customWidth="1" style="6" min="1" max="1"/>
@@ -542,11 +542,6 @@
           <t>תעתיק</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>מילה מנוקדת</t>
-        </is>
-      </c>
     </row>
     <row r="2" ht="18" customHeight="1" s="6">
       <c r="A2" s="2" t="n">
@@ -572,11 +567,6 @@
           <t>מרחבא</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>مَرْحَبًا</t>
-        </is>
-      </c>
     </row>
     <row r="3" ht="18" customHeight="1" s="6">
       <c r="A3" s="2" t="n">
@@ -602,11 +592,6 @@
           <t>אהלא</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>أَهْلًا</t>
-        </is>
-      </c>
     </row>
     <row r="4" ht="18" customHeight="1" s="6">
       <c r="A4" s="2" t="n">
@@ -632,11 +617,6 @@
           <t>אלסלאמ עליכמ</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>اَلسَّلَامُ عَلَيْكُمْ</t>
-        </is>
-      </c>
     </row>
     <row r="5" ht="18" customHeight="1" s="6">
       <c r="A5" s="2" t="n">
@@ -662,11 +642,6 @@
           <t>ודאעא</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>وَدَاعًا</t>
-        </is>
-      </c>
     </row>
     <row r="6" ht="18" customHeight="1" s="6">
       <c r="A6" s="2" t="n">
@@ -692,11 +667,6 @@
           <t>מע אלסלאמה</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>مَعَ السَّلَامَة</t>
-        </is>
-      </c>
     </row>
     <row r="7" ht="18" customHeight="1" s="6">
       <c r="A7" s="2" t="n">
@@ -722,11 +692,6 @@
           <t>נעמ</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>نَعَمْ</t>
-        </is>
-      </c>
     </row>
     <row r="8" ht="18" customHeight="1" s="6">
       <c r="A8" s="2" t="n">
@@ -752,11 +717,6 @@
           <t>לא</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>لَا</t>
-        </is>
-      </c>
     </row>
     <row r="9" ht="18" customHeight="1" s="6">
       <c r="A9" s="2" t="n">
@@ -782,11 +742,6 @@
           <t>מנ פדלכ</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>مِنْ فَضْلِكَ</t>
-        </is>
-      </c>
     </row>
     <row r="10" ht="18" customHeight="1" s="6">
       <c r="A10" s="2" t="n">
@@ -812,11 +767,6 @@
           <t>שכרא</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>شُكْرًا</t>
-        </is>
-      </c>
     </row>
     <row r="11" ht="18" customHeight="1" s="6">
       <c r="A11" s="2" t="n">
@@ -842,11 +792,6 @@
           <t>עפוא</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>عَفْوًا</t>
-        </is>
-      </c>
     </row>
     <row r="12" ht="18" customHeight="1" s="6">
       <c r="A12" s="2" t="n">
@@ -872,11 +817,6 @@
           <t>אספ</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>آسِف</t>
-        </is>
-      </c>
     </row>
     <row r="13" ht="18" customHeight="1" s="6">
       <c r="A13" s="2" t="n">
@@ -902,11 +842,6 @@
           <t>צבאח אלח'יר</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>صَبَاحُ الْخَير</t>
-        </is>
-      </c>
     </row>
     <row r="14" ht="18" customHeight="1" s="6">
       <c r="A14" s="2" t="n">
@@ -932,11 +867,6 @@
           <t>מסאא אלח'יר</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>مَسَاءُ الْخَير</t>
-        </is>
-      </c>
     </row>
     <row r="15" ht="18" customHeight="1" s="6">
       <c r="A15" s="2" t="n">
@@ -962,11 +892,6 @@
           <t>תצבח עלא ח'יר</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>تُصْبِحُ عَلَى خَيْر</t>
-        </is>
-      </c>
     </row>
     <row r="16" ht="18" customHeight="1" s="6">
       <c r="A16" s="2" t="n">
@@ -992,11 +917,6 @@
           <t>כיפ חאלכ</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>كَيْفَ حَالُكَ</t>
-        </is>
-      </c>
     </row>
     <row r="17" ht="18" customHeight="1" s="6">
       <c r="A17" s="2" t="n">
@@ -1022,11 +942,6 @@
           <t>בח'יר</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>بِخَيْر</t>
-        </is>
-      </c>
     </row>
     <row r="18" ht="18" customHeight="1" s="6">
       <c r="A18" s="2" t="n">
@@ -1052,11 +967,6 @@
           <t>מא אסמכ</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>مَا اسْمُكَ</t>
-        </is>
-      </c>
     </row>
     <row r="19" ht="18" customHeight="1" s="6">
       <c r="A19" s="2" t="n">
@@ -1082,11 +992,6 @@
           <t>אסמי</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>اِسْمِي</t>
-        </is>
-      </c>
     </row>
     <row r="20" ht="18" customHeight="1" s="6">
       <c r="A20" s="2" t="n">
@@ -1112,11 +1017,6 @@
           <t>מנ</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>مَنْ</t>
-        </is>
-      </c>
     </row>
     <row r="21" ht="18" customHeight="1" s="6">
       <c r="A21" s="2" t="n">
@@ -1142,11 +1042,6 @@
           <t>מאד'א</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>مَاذَا</t>
-        </is>
-      </c>
     </row>
     <row r="22" ht="18" customHeight="1" s="6">
       <c r="A22" s="2" t="n">
@@ -1172,11 +1067,6 @@
           <t>אינ</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>أَيْنَ</t>
-        </is>
-      </c>
     </row>
     <row r="23" ht="18" customHeight="1" s="6">
       <c r="A23" s="2" t="n">
@@ -1202,11 +1092,6 @@
           <t>מתא</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>مَتَى</t>
-        </is>
-      </c>
     </row>
     <row r="24" ht="18" customHeight="1" s="6">
       <c r="A24" s="2" t="n">
@@ -1232,11 +1117,6 @@
           <t>למאד'א</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>لِمَاذَا</t>
-        </is>
-      </c>
     </row>
     <row r="25" ht="18" customHeight="1" s="6">
       <c r="A25" s="2" t="n">
@@ -1262,11 +1142,6 @@
           <t>כיפ</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>كَيْفَ</t>
-        </is>
-      </c>
     </row>
     <row r="26" ht="18" customHeight="1" s="6">
       <c r="A26" s="2" t="n">
@@ -1292,11 +1167,6 @@
           <t>כמ</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>كَمْ</t>
-        </is>
-      </c>
     </row>
     <row r="27" ht="18" customHeight="1" s="6">
       <c r="A27" s="2" t="n">
@@ -1322,11 +1192,6 @@
           <t>אי</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>أَيّ</t>
-        </is>
-      </c>
     </row>
     <row r="28" ht="18" customHeight="1" s="6">
       <c r="A28" s="2" t="n">
@@ -1352,11 +1217,6 @@
           <t>הל</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>هَلْ</t>
-        </is>
-      </c>
     </row>
     <row r="29" ht="18" customHeight="1" s="6">
       <c r="A29" s="2" t="n">
@@ -1382,11 +1242,6 @@
           <t>ו</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>وَ</t>
-        </is>
-      </c>
     </row>
     <row r="30" ht="18" customHeight="1" s="6">
       <c r="A30" s="2" t="n">
@@ -1412,11 +1267,6 @@
           <t>או</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>أَوْ</t>
-        </is>
-      </c>
     </row>
     <row r="31" ht="18" customHeight="1" s="6">
       <c r="A31" s="2" t="n">
@@ -1442,11 +1292,6 @@
           <t>לכנ</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>لَكِنْ</t>
-        </is>
-      </c>
     </row>
     <row r="32" ht="18" customHeight="1" s="6">
       <c r="A32" s="2" t="n">
@@ -1472,11 +1317,6 @@
           <t>כמאנ</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>كَمَان</t>
-        </is>
-      </c>
     </row>
     <row r="33" ht="18" customHeight="1" s="6">
       <c r="A33" s="2" t="n">
@@ -1502,11 +1342,6 @@
           <t>אלאנ</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>اَلْآنَ</t>
-        </is>
-      </c>
     </row>
     <row r="34" ht="18" customHeight="1" s="6">
       <c r="A34" s="2" t="n">
@@ -1532,11 +1367,6 @@
           <t>הנא</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>هُنَا</t>
-        </is>
-      </c>
     </row>
     <row r="35" ht="18" customHeight="1" s="6">
       <c r="A35" s="2" t="n">
@@ -1562,11 +1392,6 @@
           <t>הנאכ</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>هُنَاكَ</t>
-        </is>
-      </c>
     </row>
     <row r="36" ht="18" customHeight="1" s="6">
       <c r="A36" s="2" t="n">
@@ -1592,11 +1417,6 @@
           <t>באלטבע/טבעאן</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>بِالطَّبْع / طَبْعًا</t>
-        </is>
-      </c>
     </row>
     <row r="37" ht="18" customHeight="1" s="6">
       <c r="A37" s="2" t="n">
@@ -1622,11 +1442,6 @@
           <t>ג'יד</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>جَيِّد</t>
-        </is>
-      </c>
     </row>
     <row r="38" ht="18" customHeight="1" s="6">
       <c r="A38" s="2" t="n">
@@ -1652,11 +1467,6 @@
           <t>סיא</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>سَيِّئ</t>
-        </is>
-      </c>
     </row>
     <row r="39" ht="18" customHeight="1" s="6">
       <c r="A39" s="2" t="n">
@@ -1682,11 +1492,6 @@
           <t>ג'דיד</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>جَدِيد</t>
-        </is>
-      </c>
     </row>
     <row r="40" ht="18" customHeight="1" s="6">
       <c r="A40" s="2" t="n">
@@ -1712,11 +1517,6 @@
           <t>קדימ</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>قَدِيم</t>
-        </is>
-      </c>
     </row>
     <row r="41" ht="18" customHeight="1" s="6">
       <c r="A41" s="2" t="n">
@@ -1740,11 +1540,6 @@
       <c r="E41" s="3" t="inlineStr">
         <is>
           <t>ערבי</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>عَرَبِيّ</t>
         </is>
       </c>
     </row>

</xml_diff>